<commit_message>
IMprove UI for journey and teams
</commit_message>
<xml_diff>
--- a/ALfred Improvement Tracker.xlsx
+++ b/ALfred Improvement Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\12985\Documents\GitHub\GREO\Alfred\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D006EE3-3483-4634-875A-AC76A257422C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32693E6-48A0-46D1-9390-5E3C35D46405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D50CF362-13FF-41C9-A62D-3420DDF519FD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="41">
   <si>
     <t>Make goals TITLE visible in tasks</t>
   </si>
@@ -105,6 +105,60 @@
   </si>
   <si>
     <t>Change the look and feel of ask for help</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Small viusal improvements. Remove emoticons</t>
+  </si>
+  <si>
+    <t>Joirney page: need ttitles</t>
+  </si>
+  <si>
+    <t>Tasks need space</t>
+  </si>
+  <si>
+    <t>Goal page need less icons, button more subtle on the side</t>
+  </si>
+  <si>
+    <t>No need for Long term anymore</t>
+  </si>
+  <si>
+    <t>I don t care aboit date in goals</t>
+  </si>
+  <si>
+    <t>My team need superfisor filter</t>
+  </si>
+  <si>
+    <t>Put links above one other,</t>
+  </si>
+  <si>
+    <t>Opportunities is a duplicate vs dev opps</t>
+  </si>
+  <si>
+    <t>Need values and achievements</t>
+  </si>
+  <si>
+    <t>Tasks</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>7. Feedback rituals</t>
+  </si>
+  <si>
+    <t>Calendar should be at the bottom of the sidebar</t>
+  </si>
+  <si>
+    <t>Sidebar</t>
+  </si>
+  <si>
+    <t>JOurney</t>
+  </si>
+  <si>
+    <t>Colors</t>
   </si>
 </sst>
 </file>
@@ -482,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DF1832-E160-45D0-A415-9BD8CDB79365}">
-  <dimension ref="B2:F21"/>
+  <dimension ref="B2:F36"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="4.36328125" customWidth="1"/>
@@ -596,6 +650,9 @@
       </c>
     </row>
     <row r="13" spans="2:6">
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
       <c r="C13" t="s">
         <v>18</v>
       </c>
@@ -608,58 +665,174 @@
     </row>
     <row r="15" spans="2:6">
       <c r="C15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6">
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4">
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4">
+      <c r="C22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4">
+      <c r="C23" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4">
+      <c r="C26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4">
+      <c r="C27" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4">
+      <c r="D28" s="1"/>
+    </row>
+    <row r="29" spans="2:4">
+      <c r="C29" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:6">
-      <c r="C16" t="s">
+    <row r="30" spans="2:4">
+      <c r="C30" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="3:4">
-      <c r="C17" t="s">
+    <row r="31" spans="2:4">
+      <c r="C31" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="3:4">
-      <c r="C18" t="s">
+    <row r="32" spans="2:4">
+      <c r="C32" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="3:4">
-      <c r="C19" t="s">
+    <row r="33" spans="3:4">
+      <c r="C33" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="3:4">
-      <c r="C20" t="s">
+    <row r="34" spans="3:4">
+      <c r="C34" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="3:4">
-      <c r="C21" t="s">
+    <row r="35" spans="3:4">
+      <c r="C35" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4">
+      <c r="C36" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update UI with improved TodoList filters and layout
</commit_message>
<xml_diff>
--- a/ALfred Improvement Tracker.xlsx
+++ b/ALfred Improvement Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\12985\Documents\GitHub\GREO\Alfred\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32693E6-48A0-46D1-9390-5E3C35D46405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FB68D30-892C-49D3-BE9F-893AE1CDBF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D50CF362-13FF-41C9-A62D-3420DDF519FD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
   <si>
     <t>Make goals TITLE visible in tasks</t>
   </si>
@@ -50,27 +50,6 @@
     <t>Make clickable the goals to get from lt to st one step at a time</t>
   </si>
   <si>
-    <t>Reactivate all nudges:</t>
-  </si>
-  <si>
-    <t>1. Compliment in the morning</t>
-  </si>
-  <si>
-    <t>2. List tasks and suggest priorities in the morning</t>
-  </si>
-  <si>
-    <t>3. invite tobthe joirnal in the evening / rituals</t>
-  </si>
-  <si>
-    <t>4. Alerts when to many tasks at the middle of the day</t>
-  </si>
-  <si>
-    <t>5. Weeklu goals setting / rituals</t>
-  </si>
-  <si>
-    <t>6. weekly coavhing session / rituals</t>
-  </si>
-  <si>
     <t>Create link to go from goals to task. It directly goes to todolist with filters</t>
   </si>
   <si>
@@ -146,9 +125,6 @@
     <t>Team</t>
   </si>
   <si>
-    <t>7. Feedback rituals</t>
-  </si>
-  <si>
     <t>Calendar should be at the bottom of the sidebar</t>
   </si>
   <si>
@@ -158,25 +134,107 @@
     <t>JOurney</t>
   </si>
   <si>
-    <t>Colors</t>
+    <t>Remove icons for supervisors, mentors and peers</t>
+  </si>
+  <si>
+    <t>Teams</t>
+  </si>
+  <si>
+    <t>Clear sidebar in tasks</t>
+  </si>
+  <si>
+    <t>Colors box</t>
+  </si>
+  <si>
+    <t>Put dates under tasks, goals on the side, copy todoist</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>Reactivate all nudges including 7 rituals</t>
+  </si>
+  <si>
+    <t>Enable multiple pages</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Sort the filter task, why is everything filtered on Caleb</t>
+  </si>
+  <si>
+    <t>Feedback page</t>
+  </si>
+  <si>
+    <t>Intelligence layer for email</t>
+  </si>
+  <si>
+    <t>Intelligence layer for task prioritization</t>
+  </si>
+  <si>
+    <t>Setting page for all triggers</t>
+  </si>
+  <si>
+    <t>Alerts when more than 5 subgoals for a group</t>
+  </si>
+  <si>
+    <t>Refresh journey based on journal</t>
+  </si>
+  <si>
+    <t>Calendar integration</t>
+  </si>
+  <si>
+    <t>Meeting not etaker</t>
+  </si>
+  <si>
+    <t>Review decks capability</t>
+  </si>
+  <si>
+    <t>Feedback</t>
+  </si>
+  <si>
+    <t>Calendar</t>
+  </si>
+  <si>
+    <t>New user onboarding</t>
+  </si>
+  <si>
+    <t>Onboarding</t>
+  </si>
+  <si>
+    <t>Task prio</t>
+  </si>
+  <si>
+    <t>Note taker</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>Deck review</t>
+  </si>
+  <si>
+    <t>5 goal max</t>
+  </si>
+  <si>
+    <t>In Trial</t>
+  </si>
+  <si>
+    <t>Enable Alfred over email</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Google Sans Text"/>
     </font>
   </fonts>
   <fills count="2">
@@ -201,7 +259,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,303 +596,420 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DF1832-E160-45D0-A415-9BD8CDB79365}">
-  <dimension ref="B2:F36"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="B2:F40"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="4.36328125" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" customWidth="1"/>
     <col min="4" max="4" width="66.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6">
-      <c r="B2" t="s">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:6">
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6">
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6">
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6">
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6">
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="2:6">
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6">
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="1" t="s">
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="2:6">
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6">
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6">
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6">
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="2:6">
-      <c r="C15" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6">
-      <c r="B16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" t="s">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C25" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C26" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="17" spans="2:4">
-      <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4">
-      <c r="B18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4">
-      <c r="C19" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4">
-      <c r="C20" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4">
-      <c r="C21" t="s">
+      <c r="D26" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" t="s">
         <v>39</v>
       </c>
-      <c r="D21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4">
-      <c r="C22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4">
-      <c r="C23" t="s">
-        <v>17</v>
-      </c>
-      <c r="D23" t="s">
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C30" t="s">
+        <v>54</v>
+      </c>
+      <c r="D30" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C31" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C32" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="24" spans="2:4">
-      <c r="C24" t="s">
-        <v>17</v>
-      </c>
-      <c r="D24" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4">
-      <c r="C26" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4">
-      <c r="C27" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4">
-      <c r="D28" s="1"/>
-    </row>
-    <row r="29" spans="2:4">
-      <c r="C29" t="s">
-        <v>16</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4">
-      <c r="C30" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4">
-      <c r="C31" t="s">
-        <v>16</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4">
-      <c r="C32" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="3:4">
+      <c r="D32" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B33" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="C33" t="s">
-        <v>16</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="3:4">
+        <v>10</v>
+      </c>
+      <c r="D33" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B34" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="C34" t="s">
-        <v>16</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" spans="3:4">
+        <v>55</v>
+      </c>
+      <c r="D34" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B35" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="C35" t="s">
-        <v>16</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="36" spans="3:4">
+        <v>40</v>
+      </c>
+      <c r="D35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B36" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="C36" t="s">
-        <v>16</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
+      </c>
+      <c r="D36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B37" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B38" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B39" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C39" t="s">
+        <v>57</v>
+      </c>
+      <c r="D39" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B40" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" t="s">
+        <v>58</v>
+      </c>
+      <c r="D40" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>